<commit_message>
Reorganize results and scoring
</commit_message>
<xml_diff>
--- a/grex/extraxted_rules/rules_neg.xlsx
+++ b/grex/extraxted_rules/rules_neg.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2" conformance="strict">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
-  <workbookPr dateCompatibility="0" defaultThemeVersion="166925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
+  <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anaal882/Documents/Courses/SDTB_project/grex/rules_results/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anaal882/Documents/GitHub/Diachronic_Treebanks_DigPhil/grex/extraxted_rules/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{D8772F19-0C49-D04C-BACB-CBE04408FDC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6A8076FC-4D1F-8441-B2AE-3432ADBC224E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5180" yWindow="3080" windowWidth="28040" windowHeight="17180" xr2:uid="{7B548511-8BA6-1C44-9B59-ABBB0DF894FA}"/>
+    <workbookView xWindow="5180" yWindow="3080" windowWidth="28040" windowHeight="17180" activeTab="1" xr2:uid="{7B548511-8BA6-1C44-9B59-ABBB0DF894FA}"/>
   </bookViews>
   <sheets>
     <sheet name="rules_neg" sheetId="1" r:id="rId1"/>
@@ -21,9 +21,6 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{79F54976-1DA5-4618-B147-4CDE4B953A38}">
-      <x14:workbookPr/>
-    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -39,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="579" uniqueCount="231">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="587" uniqueCount="237">
   <si>
     <t>Scope</t>
   </si>
@@ -644,9 +641,6 @@
     <t>1900_1950</t>
   </si>
   <si>
-    <t>ent_id: 1900_1950_344_sec397 | rules: sentence:meta:period=1900_1950, node:Y:own:has_child=No, node:X:own:Mood=Ind, node:X:own:Tense=Pres, node:X:own:Voice=Act, node:X:child:Case={'Nom'}, node:X:child:Definite={'Def', 'Ind'}, node:X:child:Degree={'Pos'}, node:X:child:Number={'Sing', 'Plur'}, node:X:child:upos={'INTJ', 'ADJ', 'PRON'}, node:X:child:rel_shallow={'nsubj', 'advcl', 'discourse', 'obj'}, node:X:child:Gender={'Neut', 'Com'}, node:X:child:PronType={'Prs'}, node:CLH:own:Mood=Ind, node:CLH:own:Tense=Pres, node:CLH:own:VerbForm=Fin, node:CLH:own:Voice=Act, node:CLH:own:upos=VERB, node:CLH:own:rel_shallow=root</t>
-  </si>
-  <si>
     <t>sent_id: 1900_1950_489_sec397 | rules: sentence:meta:period=1900_1950, node:Y:own:has_child=No, node:X:own:Mood=Ind, node:X:own:Tense=Pres, node:X:own:Voice=Act, node:X:child:Definite={'Def'}, node:X:child:Gender={'Neut'}, node:X:child:Number={'Sing'}, node:X:child:PronType={'Prs'}, node:X:child:upos={'NOUN', 'SCONJ', 'ADP', 'PRON'}, node:X:child:rel_shallow={'nsubj', 'mark', 'obj'}, node:X:child:Case={'Nom'}, node:CLH:own:Case=Nom, node:CLH:own:Definite=Ind, node:CLH:own:Degree=Pos, node:CLH:own:Gender=Com, node:CLH:own:Number=Sing, node:CLH:own:upos=ADJ, node:CLH:own:rel_shallow=root</t>
   </si>
   <si>
@@ -732,13 +726,34 @@
   </si>
   <si>
     <t>sent_id: 1700_1749_649_sec25 | rules: sentence:meta:period=1700_1749, node:Y:own:has_child=No, node:X:own:Mood=Ind, node:X:own:Tense=Pres, node:X:own:Voice=Pass, node:X:child:Case={'Nom'}, node:X:child:Definite={'Def', 'Ind'}, node:X:child:Gender={'Neut', 'Com'}, node:X:child:Number={'Sing'}, node:X:child:upos={'NOUN', 'SCONJ', 'PRON'}, node:X:child:rel_shallow={'conj', 'nsubj:pass', 'mark', 'obj'}, node:X:child:PronType={'Prs'}, node:CLH:own:Case=Nom, node:CLH:own:Definite=Ind, node:CLH:own:Degree=Pos, node:CLH:own:Gender=Com, node:CLH:own:Number=Sing, node:CLH:own:upos=ADJ, node:CLH:own:rel_shallow=root</t>
+  </si>
+  <si>
+    <t>Treebank</t>
+  </si>
+  <si>
+    <t>Sentences</t>
+  </si>
+  <si>
+    <t>Sw_Tal 1970s</t>
+  </si>
+  <si>
+    <t>6,038 </t>
+  </si>
+  <si>
+    <t>Sw_LinES</t>
+  </si>
+  <si>
+    <t>5,696 </t>
+  </si>
+  <si>
+    <t>sent_id: 1900_1950_344_sec397 | rules: sentence:meta:period=1900_1950, node:Y:own:has_child=No, node:X:own:Mood=Ind, node:X:own:Tense=Pres, node:X:own:Voice=Act, node:X:child:Case={'Nom'}, node:X:child:Definite={'Def', 'Ind'}, node:X:child:Degree={'Pos'}, node:X:child:Number={'Sing', 'Plur'}, node:X:child:upos={'INTJ', 'ADJ', 'PRON'}, node:X:child:rel_shallow={'nsubj', 'advcl', 'discourse', 'obj'}, node:X:child:Gender={'Neut', 'Com'}, node:X:child:PronType={'Prs'}, node:CLH:own:Mood=Ind, node:CLH:own:Tense=Pres, node:CLH:own:VerbForm=Fin, node:CLH:own:Voice=Act, node:CLH:own:upos=VERB, node:CLH:own:rel_shallow=root</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="19" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="21">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -878,6 +893,17 @@
       <sz val="18"/>
       <color theme="1"/>
       <name val="Calibri (Body)"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="1"/>
+      <name val=".AppleSystemUIFont"/>
+    </font>
+    <font>
+      <sz val="13"/>
+      <color theme="1"/>
+      <name val=".AppleSystemUIFont"/>
     </font>
   </fonts>
   <fills count="35">
@@ -1075,15 +1101,15 @@
   </fills>
   <borders count="11">
     <border>
-      <start/>
-      <end/>
+      <left/>
+      <right/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
     <border>
-      <start/>
-      <end/>
+      <left/>
+      <right/>
       <top/>
       <bottom style="thick">
         <color theme="4"/>
@@ -1091,8 +1117,8 @@
       <diagonal/>
     </border>
     <border>
-      <start/>
-      <end/>
+      <left/>
+      <right/>
       <top/>
       <bottom style="thick">
         <color theme="4" tint="0.499984740745262"/>
@@ -1100,8 +1126,8 @@
       <diagonal/>
     </border>
     <border>
-      <start/>
-      <end/>
+      <left/>
+      <right/>
       <top/>
       <bottom style="medium">
         <color theme="4" tint="0.39997558519241921"/>
@@ -1109,12 +1135,12 @@
       <diagonal/>
     </border>
     <border>
-      <start style="thin">
+      <left style="thin">
         <color rgb="FF7F7F7F"/>
-      </start>
-      <end style="thin">
+      </left>
+      <right style="thin">
         <color rgb="FF7F7F7F"/>
-      </end>
+      </right>
       <top style="thin">
         <color rgb="FF7F7F7F"/>
       </top>
@@ -1124,12 +1150,12 @@
       <diagonal/>
     </border>
     <border>
-      <start style="thin">
+      <left style="thin">
         <color rgb="FF3F3F3F"/>
-      </start>
-      <end style="thin">
+      </left>
+      <right style="thin">
         <color rgb="FF3F3F3F"/>
-      </end>
+      </right>
       <top style="thin">
         <color rgb="FF3F3F3F"/>
       </top>
@@ -1139,8 +1165,8 @@
       <diagonal/>
     </border>
     <border>
-      <start/>
-      <end/>
+      <left/>
+      <right/>
       <top/>
       <bottom style="double">
         <color rgb="FFFF8001"/>
@@ -1148,12 +1174,12 @@
       <diagonal/>
     </border>
     <border>
-      <start style="double">
+      <left style="double">
         <color rgb="FF3F3F3F"/>
-      </start>
-      <end style="double">
+      </left>
+      <right style="double">
         <color rgb="FF3F3F3F"/>
-      </end>
+      </right>
       <top style="double">
         <color rgb="FF3F3F3F"/>
       </top>
@@ -1163,12 +1189,12 @@
       <diagonal/>
     </border>
     <border>
-      <start style="thin">
+      <left style="thin">
         <color rgb="FFB2B2B2"/>
-      </start>
-      <end style="thin">
+      </left>
+      <right style="thin">
         <color rgb="FFB2B2B2"/>
-      </end>
+      </right>
       <top style="thin">
         <color rgb="FFB2B2B2"/>
       </top>
@@ -1178,8 +1204,8 @@
       <diagonal/>
     </border>
     <border>
-      <start/>
-      <end/>
+      <left/>
+      <right/>
       <top style="thin">
         <color theme="4"/>
       </top>
@@ -1189,12 +1215,12 @@
       <diagonal/>
     </border>
     <border>
-      <start style="thin">
+      <left style="thin">
         <color indexed="64"/>
-      </start>
-      <end style="thin">
+      </left>
+      <right style="thin">
         <color indexed="64"/>
-      </end>
+      </right>
       <top style="thin">
         <color indexed="64"/>
       </top>
@@ -1248,17 +1274,19 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1318,7 +1346,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://purl.oclc.org/ooxml/drawingml/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1471,25 +1499,25 @@
         </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
-            <a:gs pos="0%">
+            <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:lumMod val="110%"/>
-                <a:satMod val="105%"/>
-                <a:tint val="67%"/>
+                <a:lumMod val="110000"/>
+                <a:satMod val="105000"/>
+                <a:tint val="67000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50%">
+            <a:gs pos="50000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105%"/>
-                <a:satMod val="103%"/>
-                <a:tint val="73%"/>
+                <a:lumMod val="105000"/>
+                <a:satMod val="103000"/>
+                <a:tint val="73000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="100%">
+            <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105%"/>
-                <a:satMod val="109%"/>
-                <a:tint val="81%"/>
+                <a:lumMod val="105000"/>
+                <a:satMod val="109000"/>
+                <a:tint val="81000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -1497,25 +1525,25 @@
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
-            <a:gs pos="0%">
+            <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:satMod val="103%"/>
-                <a:lumMod val="102%"/>
-                <a:tint val="94%"/>
+                <a:satMod val="103000"/>
+                <a:lumMod val="102000"/>
+                <a:tint val="94000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50%">
+            <a:gs pos="50000">
               <a:schemeClr val="phClr">
-                <a:satMod val="110%"/>
-                <a:lumMod val="100%"/>
-                <a:shade val="100%"/>
+                <a:satMod val="110000"/>
+                <a:lumMod val="100000"/>
+                <a:shade val="100000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="100%">
+            <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="99%"/>
-                <a:satMod val="120%"/>
-                <a:shade val="78%"/>
+                <a:lumMod val="99000"/>
+                <a:satMod val="120000"/>
+                <a:shade val="78000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -1528,21 +1556,21 @@
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800%"/>
+          <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800%"/>
+          <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800%"/>
+          <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
@@ -1556,7 +1584,7 @@
           <a:effectLst>
             <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
               <a:srgbClr val="000000">
-                <a:alpha val="63%"/>
+                <a:alpha val="63000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
@@ -1568,32 +1596,32 @@
         </a:solidFill>
         <a:solidFill>
           <a:schemeClr val="phClr">
-            <a:tint val="95%"/>
-            <a:satMod val="170%"/>
+            <a:tint val="95000"/>
+            <a:satMod val="170000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
-            <a:gs pos="0%">
+            <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="93%"/>
-                <a:satMod val="150%"/>
-                <a:shade val="98%"/>
-                <a:lumMod val="102%"/>
+                <a:tint val="93000"/>
+                <a:satMod val="150000"/>
+                <a:shade val="98000"/>
+                <a:lumMod val="102000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50%">
+            <a:gs pos="50000">
               <a:schemeClr val="phClr">
-                <a:tint val="98%"/>
-                <a:satMod val="130%"/>
-                <a:shade val="90%"/>
-                <a:lumMod val="103%"/>
+                <a:tint val="98000"/>
+                <a:satMod val="130000"/>
+                <a:shade val="90000"/>
+                <a:lumMod val="103000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="100%">
+            <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="63%"/>
-                <a:satMod val="120%"/>
+                <a:shade val="63000"/>
+                <a:satMod val="120000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -1613,38 +1641,38 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9DBFE486-2B5C-2644-93C1-DE36ADFD1FEE}">
-  <dimension ref="A1:I184"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9DBFE486-2B5C-2644-93C1-DE36ADFD1FEE}">
+  <dimension ref="A1:N184"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="79.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:14">
+      <c r="A1" s="6" t="s">
         <v>195</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
-      <c r="H1" s="3"/>
-      <c r="I1" s="3"/>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A2" s="3"/>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
-      <c r="I2" s="3"/>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
+      <c r="H1" s="7"/>
+      <c r="I1" s="7"/>
+    </row>
+    <row r="2" spans="1:14">
+      <c r="A2" s="7"/>
+      <c r="B2" s="7"/>
+      <c r="C2" s="7"/>
+      <c r="D2" s="7"/>
+      <c r="E2" s="7"/>
+      <c r="F2" s="7"/>
+      <c r="G2" s="7"/>
+      <c r="H2" s="7"/>
+      <c r="I2" s="7"/>
+    </row>
+    <row r="3" spans="1:14">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -1652,7 +1680,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:14">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -1660,53 +1688,53 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:14">
       <c r="A5" t="s">
         <v>4</v>
       </c>
       <c r="B5">
         <v>448</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="3" t="s">
         <v>196</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="F5" s="5" t="s">
+      <c r="F5" s="3" t="s">
         <v>198</v>
       </c>
-      <c r="G5" s="5" t="s">
+      <c r="G5" s="3" t="s">
         <v>199</v>
       </c>
-      <c r="H5" s="5" t="s">
+      <c r="H5" s="3" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:14">
       <c r="A6" t="s">
         <v>5</v>
       </c>
       <c r="B6">
         <v>30</v>
       </c>
-      <c r="D6" s="5">
+      <c r="D6" s="3">
         <v>6</v>
       </c>
-      <c r="E6" s="5">
+      <c r="E6" s="3">
         <v>11</v>
       </c>
-      <c r="F6" s="5">
+      <c r="F6" s="3">
         <v>5</v>
       </c>
-      <c r="G6" s="5">
+      <c r="G6" s="3">
         <v>3</v>
       </c>
-      <c r="H6" s="5">
+      <c r="H6" s="3">
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:14" ht="17">
       <c r="A8" t="s">
         <v>6</v>
       </c>
@@ -1734,8 +1762,20 @@
       <c r="I8" t="s">
         <v>194</v>
       </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="K8" s="4" t="s">
+        <v>230</v>
+      </c>
+      <c r="L8" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="M8" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N8" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" ht="17">
       <c r="A9" s="1" t="s">
         <v>14</v>
       </c>
@@ -1763,8 +1803,20 @@
       <c r="I9" s="1">
         <v>1.1779999999999999</v>
       </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="K9" s="5" t="s">
+        <v>232</v>
+      </c>
+      <c r="L9" s="5" t="s">
+        <v>233</v>
+      </c>
+      <c r="M9" s="5">
+        <v>58</v>
+      </c>
+      <c r="N9" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" ht="17">
       <c r="A10" s="1" t="s">
         <v>17</v>
       </c>
@@ -1792,8 +1844,20 @@
       <c r="I10" s="1">
         <v>1.0149999999999999</v>
       </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="K10" s="5" t="s">
+        <v>234</v>
+      </c>
+      <c r="L10" s="5" t="s">
+        <v>235</v>
+      </c>
+      <c r="M10" s="5">
+        <v>75</v>
+      </c>
+      <c r="N10" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14">
       <c r="A11" s="1" t="s">
         <v>18</v>
       </c>
@@ -1822,7 +1886,7 @@
         <v>1.0149999999999999</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:14">
       <c r="A12" s="1" t="s">
         <v>19</v>
       </c>
@@ -1851,7 +1915,7 @@
         <v>1.0149999999999999</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:14">
       <c r="A13" s="1" t="s">
         <v>20</v>
       </c>
@@ -1880,7 +1944,7 @@
         <v>0.94899999999999995</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:14">
       <c r="A14" s="1" t="s">
         <v>21</v>
       </c>
@@ -1909,7 +1973,7 @@
         <v>0.94899999999999995</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:14">
       <c r="A15" s="1" t="s">
         <v>23</v>
       </c>
@@ -1938,7 +2002,7 @@
         <v>0.94899999999999995</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:14">
       <c r="A16" s="1" t="s">
         <v>24</v>
       </c>
@@ -1967,7 +2031,7 @@
         <v>0.88900000000000001</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:9">
       <c r="A17" s="1" t="s">
         <v>25</v>
       </c>
@@ -1996,7 +2060,7 @@
         <v>0.70499999999999996</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:9">
       <c r="A18" s="1" t="s">
         <v>26</v>
       </c>
@@ -2025,7 +2089,7 @@
         <v>0.66900000000000004</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:9">
       <c r="A19" s="1" t="s">
         <v>27</v>
       </c>
@@ -2054,7 +2118,7 @@
         <v>0.63500000000000001</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:9">
       <c r="A20" s="1" t="s">
         <v>28</v>
       </c>
@@ -2083,7 +2147,7 @@
         <v>0.63500000000000001</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:9">
       <c r="A21" s="1" t="s">
         <v>29</v>
       </c>
@@ -2112,7 +2176,7 @@
         <v>0.57499999999999996</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:9">
       <c r="A22" s="1" t="s">
         <v>30</v>
       </c>
@@ -2141,7 +2205,7 @@
         <v>0.57499999999999996</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:9">
       <c r="A23" s="1" t="s">
         <v>31</v>
       </c>
@@ -2170,7 +2234,7 @@
         <v>0.57499999999999996</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:9">
       <c r="A24" s="1" t="s">
         <v>32</v>
       </c>
@@ -2199,7 +2263,7 @@
         <v>0.57499999999999996</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:9">
       <c r="A25" s="1" t="s">
         <v>33</v>
       </c>
@@ -2228,7 +2292,7 @@
         <v>0.53</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:9">
       <c r="A26" s="1" t="s">
         <v>34</v>
       </c>
@@ -2257,7 +2321,7 @@
         <v>0.51700000000000002</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:9">
       <c r="A27" s="1" t="s">
         <v>35</v>
       </c>
@@ -2286,7 +2350,7 @@
         <v>0.51700000000000002</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:9">
       <c r="A28" s="1" t="s">
         <v>36</v>
       </c>
@@ -2315,7 +2379,7 @@
         <v>0.51400000000000001</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:9">
       <c r="A29" s="1" t="s">
         <v>37</v>
       </c>
@@ -2344,7 +2408,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:9">
       <c r="A30" s="1" t="s">
         <v>38</v>
       </c>
@@ -2373,7 +2437,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:9">
       <c r="A31" s="1" t="s">
         <v>39</v>
       </c>
@@ -2402,7 +2466,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:9">
       <c r="A32" s="1" t="s">
         <v>40</v>
       </c>
@@ -2431,7 +2495,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:9">
       <c r="A33" s="1" t="s">
         <v>41</v>
       </c>
@@ -2460,7 +2524,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:9">
       <c r="A34" s="1" t="s">
         <v>42</v>
       </c>
@@ -2489,7 +2553,7 @@
         <v>0.46100000000000002</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:9">
       <c r="A35" s="1" t="s">
         <v>43</v>
       </c>
@@ -2518,7 +2582,7 @@
         <v>0.438</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:9">
       <c r="A36" s="1" t="s">
         <v>44</v>
       </c>
@@ -2547,7 +2611,7 @@
         <v>0.438</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:9">
       <c r="A37" s="1" t="s">
         <v>45</v>
       </c>
@@ -2576,7 +2640,7 @@
         <v>0.40699999999999997</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:9">
       <c r="A38" s="1" t="s">
         <v>46</v>
       </c>
@@ -2605,7 +2669,7 @@
         <v>0.40200000000000002</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:9">
       <c r="A39" s="1" t="s">
         <v>47</v>
       </c>
@@ -2634,7 +2698,7 @@
         <v>0.40200000000000002</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:9">
       <c r="A40" s="1" t="s">
         <v>48</v>
       </c>
@@ -2663,7 +2727,7 @@
         <v>0.38500000000000001</v>
       </c>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:9">
       <c r="A41" s="1" t="s">
         <v>49</v>
       </c>
@@ -2692,7 +2756,7 @@
         <v>0.38500000000000001</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:9">
       <c r="A42" s="1" t="s">
         <v>50</v>
       </c>
@@ -2721,7 +2785,7 @@
         <v>0.373</v>
       </c>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:9">
       <c r="A43" s="2" t="s">
         <v>106</v>
       </c>
@@ -2750,7 +2814,7 @@
         <v>0.372</v>
       </c>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:9">
       <c r="A44" s="2" t="s">
         <v>107</v>
       </c>
@@ -2779,7 +2843,7 @@
         <v>0.372</v>
       </c>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:9">
       <c r="A45" s="2" t="s">
         <v>108</v>
       </c>
@@ -2808,7 +2872,7 @@
         <v>0.372</v>
       </c>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:9">
       <c r="A46" s="2" t="s">
         <v>109</v>
       </c>
@@ -2837,7 +2901,7 @@
         <v>0.372</v>
       </c>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:9">
       <c r="A47" s="2" t="s">
         <v>110</v>
       </c>
@@ -2866,7 +2930,7 @@
         <v>0.372</v>
       </c>
     </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:9">
       <c r="A48" s="2" t="s">
         <v>111</v>
       </c>
@@ -2895,7 +2959,7 @@
         <v>0.372</v>
       </c>
     </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:9">
       <c r="A49" s="2" t="s">
         <v>112</v>
       </c>
@@ -2924,7 +2988,7 @@
         <v>0.372</v>
       </c>
     </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:9">
       <c r="A50" s="2" t="s">
         <v>113</v>
       </c>
@@ -2953,7 +3017,7 @@
         <v>0.372</v>
       </c>
     </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:9">
       <c r="A51" s="2" t="s">
         <v>114</v>
       </c>
@@ -2982,7 +3046,7 @@
         <v>0.372</v>
       </c>
     </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:9">
       <c r="A52" s="2" t="s">
         <v>115</v>
       </c>
@@ -3011,7 +3075,7 @@
         <v>0.372</v>
       </c>
     </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:9">
       <c r="A53" s="2" t="s">
         <v>116</v>
       </c>
@@ -3040,7 +3104,7 @@
         <v>0.372</v>
       </c>
     </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:9">
       <c r="A54" s="2" t="s">
         <v>117</v>
       </c>
@@ -3069,7 +3133,7 @@
         <v>0.372</v>
       </c>
     </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:9">
       <c r="A55" s="2" t="s">
         <v>118</v>
       </c>
@@ -3098,7 +3162,7 @@
         <v>0.372</v>
       </c>
     </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:9">
       <c r="A56" s="2" t="s">
         <v>119</v>
       </c>
@@ -3127,7 +3191,7 @@
         <v>0.372</v>
       </c>
     </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:9">
       <c r="A57" s="2" t="s">
         <v>120</v>
       </c>
@@ -3156,7 +3220,7 @@
         <v>0.372</v>
       </c>
     </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:9">
       <c r="A58" s="2" t="s">
         <v>121</v>
       </c>
@@ -3185,7 +3249,7 @@
         <v>0.372</v>
       </c>
     </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:9">
       <c r="A59" s="2" t="s">
         <v>122</v>
       </c>
@@ -3214,7 +3278,7 @@
         <v>0.372</v>
       </c>
     </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:9">
       <c r="A60" s="2" t="s">
         <v>123</v>
       </c>
@@ -3243,7 +3307,7 @@
         <v>0.372</v>
       </c>
     </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:9">
       <c r="A61" s="2" t="s">
         <v>124</v>
       </c>
@@ -3272,7 +3336,7 @@
         <v>0.372</v>
       </c>
     </row>
-    <row r="62" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:9">
       <c r="A62" s="2" t="s">
         <v>125</v>
       </c>
@@ -3301,7 +3365,7 @@
         <v>0.372</v>
       </c>
     </row>
-    <row r="63" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:9">
       <c r="A63" s="2" t="s">
         <v>126</v>
       </c>
@@ -3330,7 +3394,7 @@
         <v>0.372</v>
       </c>
     </row>
-    <row r="64" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:9">
       <c r="A64" s="2" t="s">
         <v>127</v>
       </c>
@@ -3359,7 +3423,7 @@
         <v>0.372</v>
       </c>
     </row>
-    <row r="65" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:9">
       <c r="A65" s="2" t="s">
         <v>128</v>
       </c>
@@ -3388,7 +3452,7 @@
         <v>0.372</v>
       </c>
     </row>
-    <row r="66" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:9">
       <c r="A66" s="2" t="s">
         <v>129</v>
       </c>
@@ -3417,7 +3481,7 @@
         <v>0.372</v>
       </c>
     </row>
-    <row r="67" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:9">
       <c r="A67" s="2" t="s">
         <v>130</v>
       </c>
@@ -3446,7 +3510,7 @@
         <v>0.372</v>
       </c>
     </row>
-    <row r="68" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:9">
       <c r="A68" s="2" t="s">
         <v>131</v>
       </c>
@@ -3475,7 +3539,7 @@
         <v>0.372</v>
       </c>
     </row>
-    <row r="69" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:9">
       <c r="A69" s="2" t="s">
         <v>132</v>
       </c>
@@ -3504,7 +3568,7 @@
         <v>0.372</v>
       </c>
     </row>
-    <row r="70" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:9">
       <c r="A70" s="2" t="s">
         <v>133</v>
       </c>
@@ -3533,7 +3597,7 @@
         <v>0.372</v>
       </c>
     </row>
-    <row r="71" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:9">
       <c r="A71" s="1" t="s">
         <v>51</v>
       </c>
@@ -3562,7 +3626,7 @@
         <v>0.36899999999999999</v>
       </c>
     </row>
-    <row r="72" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:9">
       <c r="A72" s="1" t="s">
         <v>52</v>
       </c>
@@ -3591,7 +3655,7 @@
         <v>0.36199999999999999</v>
       </c>
     </row>
-    <row r="73" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:9">
       <c r="A73" s="1" t="s">
         <v>53</v>
       </c>
@@ -3620,7 +3684,7 @@
         <v>0.34</v>
       </c>
     </row>
-    <row r="74" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:9">
       <c r="A74" s="1" t="s">
         <v>54</v>
       </c>
@@ -3649,7 +3713,7 @@
         <v>0.34</v>
       </c>
     </row>
-    <row r="75" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:9">
       <c r="A75" s="1" t="s">
         <v>55</v>
       </c>
@@ -3678,7 +3742,7 @@
         <v>0.32</v>
       </c>
     </row>
-    <row r="76" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:9">
       <c r="A76" s="1" t="s">
         <v>56</v>
       </c>
@@ -3707,7 +3771,7 @@
         <v>0.308</v>
       </c>
     </row>
-    <row r="77" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:9">
       <c r="A77" s="1" t="s">
         <v>57</v>
       </c>
@@ -3736,7 +3800,7 @@
         <v>0.29699999999999999</v>
       </c>
     </row>
-    <row r="78" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:9">
       <c r="A78" s="1" t="s">
         <v>58</v>
       </c>
@@ -3765,7 +3829,7 @@
         <v>0.29399999999999998</v>
       </c>
     </row>
-    <row r="79" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:9">
       <c r="A79" s="1" t="s">
         <v>59</v>
       </c>
@@ -3794,7 +3858,7 @@
         <v>0.28000000000000003</v>
       </c>
     </row>
-    <row r="80" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:9">
       <c r="A80" s="1" t="s">
         <v>60</v>
       </c>
@@ -3823,7 +3887,7 @@
         <v>0.26</v>
       </c>
     </row>
-    <row r="81" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:9">
       <c r="A81" s="2" t="s">
         <v>134</v>
       </c>
@@ -3852,7 +3916,7 @@
         <v>0.26</v>
       </c>
     </row>
-    <row r="82" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:9">
       <c r="A82" s="1" t="s">
         <v>61</v>
       </c>
@@ -3881,7 +3945,7 @@
         <v>0.25900000000000001</v>
       </c>
     </row>
-    <row r="83" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:9">
       <c r="A83" s="2" t="s">
         <v>135</v>
       </c>
@@ -3910,7 +3974,7 @@
         <v>0.255</v>
       </c>
     </row>
-    <row r="84" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:9">
       <c r="A84" s="1" t="s">
         <v>62</v>
       </c>
@@ -3939,7 +4003,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="85" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:9">
       <c r="A85" s="1" t="s">
         <v>63</v>
       </c>
@@ -3968,7 +4032,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="86" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:9">
       <c r="A86" s="2" t="s">
         <v>136</v>
       </c>
@@ -3997,7 +4061,7 @@
         <v>0.246</v>
       </c>
     </row>
-    <row r="87" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:9">
       <c r="A87" s="2" t="s">
         <v>137</v>
       </c>
@@ -4026,7 +4090,7 @@
         <v>0.24</v>
       </c>
     </row>
-    <row r="88" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:9">
       <c r="A88" s="2" t="s">
         <v>138</v>
       </c>
@@ -4055,7 +4119,7 @@
         <v>0.23899999999999999</v>
       </c>
     </row>
-    <row r="89" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:9">
       <c r="A89" s="1" t="s">
         <v>64</v>
       </c>
@@ -4084,7 +4148,7 @@
         <v>0.23</v>
       </c>
     </row>
-    <row r="90" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:9">
       <c r="A90" s="1" t="s">
         <v>65</v>
       </c>
@@ -4113,7 +4177,7 @@
         <v>0.22700000000000001</v>
       </c>
     </row>
-    <row r="91" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:9">
       <c r="A91" s="2" t="s">
         <v>139</v>
       </c>
@@ -4142,7 +4206,7 @@
         <v>0.223</v>
       </c>
     </row>
-    <row r="92" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:9">
       <c r="A92" s="1" t="s">
         <v>66</v>
       </c>
@@ -4171,7 +4235,7 @@
         <v>0.222</v>
       </c>
     </row>
-    <row r="93" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:9">
       <c r="A93" s="2" t="s">
         <v>140</v>
       </c>
@@ -4200,7 +4264,7 @@
         <v>0.221</v>
       </c>
     </row>
-    <row r="94" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:9">
       <c r="A94" s="2" t="s">
         <v>141</v>
       </c>
@@ -4229,7 +4293,7 @@
         <v>0.221</v>
       </c>
     </row>
-    <row r="95" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:9">
       <c r="A95" s="1" t="s">
         <v>67</v>
       </c>
@@ -4258,7 +4322,7 @@
         <v>0.20899999999999999</v>
       </c>
     </row>
-    <row r="96" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:9">
       <c r="A96" s="1" t="s">
         <v>68</v>
       </c>
@@ -4287,7 +4351,7 @@
         <v>0.20899999999999999</v>
       </c>
     </row>
-    <row r="97" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:9">
       <c r="A97" s="1" t="s">
         <v>69</v>
       </c>
@@ -4316,7 +4380,7 @@
         <v>0.20899999999999999</v>
       </c>
     </row>
-    <row r="98" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:9">
       <c r="A98" s="2" t="s">
         <v>142</v>
       </c>
@@ -4345,7 +4409,7 @@
         <v>0.191</v>
       </c>
     </row>
-    <row r="99" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:9">
       <c r="A99" s="2" t="s">
         <v>143</v>
       </c>
@@ -4374,7 +4438,7 @@
         <v>0.188</v>
       </c>
     </row>
-    <row r="100" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:9">
       <c r="A100" s="2" t="s">
         <v>144</v>
       </c>
@@ -4403,7 +4467,7 @@
         <v>0.188</v>
       </c>
     </row>
-    <row r="101" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:9">
       <c r="A101" s="2" t="s">
         <v>145</v>
       </c>
@@ -4432,7 +4496,7 @@
         <v>0.188</v>
       </c>
     </row>
-    <row r="102" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:9">
       <c r="A102" s="2" t="s">
         <v>146</v>
       </c>
@@ -4461,7 +4525,7 @@
         <v>0.188</v>
       </c>
     </row>
-    <row r="103" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:9">
       <c r="A103" s="1" t="s">
         <v>70</v>
       </c>
@@ -4490,7 +4554,7 @@
         <v>0.184</v>
       </c>
     </row>
-    <row r="104" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:9">
       <c r="A104" s="1" t="s">
         <v>71</v>
       </c>
@@ -4519,7 +4583,7 @@
         <v>0.183</v>
       </c>
     </row>
-    <row r="105" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:9">
       <c r="A105" s="1" t="s">
         <v>72</v>
       </c>
@@ -4548,7 +4612,7 @@
         <v>0.18</v>
       </c>
     </row>
-    <row r="106" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:9">
       <c r="A106" s="1" t="s">
         <v>73</v>
       </c>
@@ -4577,7 +4641,7 @@
         <v>0.17899999999999999</v>
       </c>
     </row>
-    <row r="107" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:9">
       <c r="A107" s="1" t="s">
         <v>74</v>
       </c>
@@ -4606,7 +4670,7 @@
         <v>0.17899999999999999</v>
       </c>
     </row>
-    <row r="108" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:9">
       <c r="A108" s="1" t="s">
         <v>75</v>
       </c>
@@ -4635,7 +4699,7 @@
         <v>0.17599999999999999</v>
       </c>
     </row>
-    <row r="109" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:9">
       <c r="A109" s="2" t="s">
         <v>147</v>
       </c>
@@ -4664,7 +4728,7 @@
         <v>0.16600000000000001</v>
       </c>
     </row>
-    <row r="110" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:9">
       <c r="A110" s="2" t="s">
         <v>148</v>
       </c>
@@ -4693,7 +4757,7 @@
         <v>0.16600000000000001</v>
       </c>
     </row>
-    <row r="111" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:9">
       <c r="A111" s="2" t="s">
         <v>149</v>
       </c>
@@ -4722,7 +4786,7 @@
         <v>0.16300000000000001</v>
       </c>
     </row>
-    <row r="112" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:9">
       <c r="A112" s="2" t="s">
         <v>150</v>
       </c>
@@ -4751,7 +4815,7 @@
         <v>0.16300000000000001</v>
       </c>
     </row>
-    <row r="113" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:9">
       <c r="A113" s="1" t="s">
         <v>76</v>
       </c>
@@ -4780,7 +4844,7 @@
         <v>0.16200000000000001</v>
       </c>
     </row>
-    <row r="114" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:9">
       <c r="A114" s="1" t="s">
         <v>77</v>
       </c>
@@ -4809,7 +4873,7 @@
         <v>0.16200000000000001</v>
       </c>
     </row>
-    <row r="115" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:9">
       <c r="A115" s="2" t="s">
         <v>151</v>
       </c>
@@ -4838,7 +4902,7 @@
         <v>0.159</v>
       </c>
     </row>
-    <row r="116" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:9">
       <c r="A116" s="1" t="s">
         <v>78</v>
       </c>
@@ -4867,7 +4931,7 @@
         <v>0.155</v>
       </c>
     </row>
-    <row r="117" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:9">
       <c r="A117" s="2" t="s">
         <v>152</v>
       </c>
@@ -4896,7 +4960,7 @@
         <v>0.154</v>
       </c>
     </row>
-    <row r="118" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:9">
       <c r="A118" s="1" t="s">
         <v>79</v>
       </c>
@@ -4925,7 +4989,7 @@
         <v>0.153</v>
       </c>
     </row>
-    <row r="119" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:9">
       <c r="A119" s="1" t="s">
         <v>80</v>
       </c>
@@ -4954,7 +5018,7 @@
         <v>0.153</v>
       </c>
     </row>
-    <row r="120" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:9">
       <c r="A120" s="2" t="s">
         <v>153</v>
       </c>
@@ -4983,7 +5047,7 @@
         <v>0.151</v>
       </c>
     </row>
-    <row r="121" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:9">
       <c r="A121" s="2" t="s">
         <v>154</v>
       </c>
@@ -5012,7 +5076,7 @@
         <v>0.151</v>
       </c>
     </row>
-    <row r="122" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:9">
       <c r="A122" s="2" t="s">
         <v>155</v>
       </c>
@@ -5041,7 +5105,7 @@
         <v>0.14799999999999999</v>
       </c>
     </row>
-    <row r="123" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:9">
       <c r="A123" s="2" t="s">
         <v>156</v>
       </c>
@@ -5070,7 +5134,7 @@
         <v>0.14799999999999999</v>
       </c>
     </row>
-    <row r="124" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:9">
       <c r="A124" s="2" t="s">
         <v>157</v>
       </c>
@@ -5099,7 +5163,7 @@
         <v>0.14399999999999999</v>
       </c>
     </row>
-    <row r="125" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:9">
       <c r="A125" s="2" t="s">
         <v>158</v>
       </c>
@@ -5128,7 +5192,7 @@
         <v>0.14399999999999999</v>
       </c>
     </row>
-    <row r="126" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:9">
       <c r="A126" s="2" t="s">
         <v>159</v>
       </c>
@@ -5157,7 +5221,7 @@
         <v>0.14299999999999999</v>
       </c>
     </row>
-    <row r="127" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:9">
       <c r="A127" s="1" t="s">
         <v>81</v>
       </c>
@@ -5186,7 +5250,7 @@
         <v>0.14199999999999999</v>
       </c>
     </row>
-    <row r="128" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:9">
       <c r="A128" s="2" t="s">
         <v>160</v>
       </c>
@@ -5215,7 +5279,7 @@
         <v>0.14099999999999999</v>
       </c>
     </row>
-    <row r="129" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:9">
       <c r="A129" s="2" t="s">
         <v>161</v>
       </c>
@@ -5244,7 +5308,7 @@
         <v>0.14000000000000001</v>
       </c>
     </row>
-    <row r="130" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:9">
       <c r="A130" s="1" t="s">
         <v>82</v>
       </c>
@@ -5273,7 +5337,7 @@
         <v>0.13900000000000001</v>
       </c>
     </row>
-    <row r="131" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:9">
       <c r="A131" s="1" t="s">
         <v>83</v>
       </c>
@@ -5302,7 +5366,7 @@
         <v>0.13800000000000001</v>
       </c>
     </row>
-    <row r="132" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:9">
       <c r="A132" s="2" t="s">
         <v>162</v>
       </c>
@@ -5331,7 +5395,7 @@
         <v>0.123</v>
       </c>
     </row>
-    <row r="133" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:9">
       <c r="A133" s="2" t="s">
         <v>163</v>
       </c>
@@ -5360,7 +5424,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="134" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:9">
       <c r="A134" s="1" t="s">
         <v>84</v>
       </c>
@@ -5389,7 +5453,7 @@
         <v>0.11899999999999999</v>
       </c>
     </row>
-    <row r="135" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:9">
       <c r="A135" s="2" t="s">
         <v>164</v>
       </c>
@@ -5418,7 +5482,7 @@
         <v>0.11799999999999999</v>
       </c>
     </row>
-    <row r="136" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:9">
       <c r="A136" s="1" t="s">
         <v>85</v>
       </c>
@@ -5447,7 +5511,7 @@
         <v>0.11600000000000001</v>
       </c>
     </row>
-    <row r="137" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:9">
       <c r="A137" s="1" t="s">
         <v>86</v>
       </c>
@@ -5476,7 +5540,7 @@
         <v>0.112</v>
       </c>
     </row>
-    <row r="138" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:9">
       <c r="A138" s="2" t="s">
         <v>165</v>
       </c>
@@ -5505,7 +5569,7 @@
         <v>0.11</v>
       </c>
     </row>
-    <row r="139" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:9">
       <c r="A139" s="2" t="s">
         <v>166</v>
       </c>
@@ -5534,7 +5598,7 @@
         <v>0.11</v>
       </c>
     </row>
-    <row r="140" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:9">
       <c r="A140" s="2" t="s">
         <v>167</v>
       </c>
@@ -5563,7 +5627,7 @@
         <v>0.11</v>
       </c>
     </row>
-    <row r="141" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:9">
       <c r="A141" s="1" t="s">
         <v>87</v>
       </c>
@@ -5592,7 +5656,7 @@
         <v>0.107</v>
       </c>
     </row>
-    <row r="142" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:9">
       <c r="A142" s="2" t="s">
         <v>168</v>
       </c>
@@ -5621,7 +5685,7 @@
         <v>0.106</v>
       </c>
     </row>
-    <row r="143" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:9">
       <c r="A143" s="2" t="s">
         <v>169</v>
       </c>
@@ -5650,7 +5714,7 @@
         <v>0.106</v>
       </c>
     </row>
-    <row r="144" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:9">
       <c r="A144" s="2" t="s">
         <v>170</v>
       </c>
@@ -5679,7 +5743,7 @@
         <v>0.10299999999999999</v>
       </c>
     </row>
-    <row r="145" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:9">
       <c r="A145" s="2" t="s">
         <v>171</v>
       </c>
@@ -5708,7 +5772,7 @@
         <v>0.10199999999999999</v>
       </c>
     </row>
-    <row r="146" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:9">
       <c r="A146" s="1" t="s">
         <v>88</v>
       </c>
@@ -5737,7 +5801,7 @@
         <v>0.10100000000000001</v>
       </c>
     </row>
-    <row r="147" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:9">
       <c r="A147" s="2" t="s">
         <v>172</v>
       </c>
@@ -5766,7 +5830,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="148" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:9">
       <c r="A148" s="1" t="s">
         <v>89</v>
       </c>
@@ -5795,7 +5859,7 @@
         <v>9.9000000000000005E-2</v>
       </c>
     </row>
-    <row r="149" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:9">
       <c r="A149" s="1" t="s">
         <v>90</v>
       </c>
@@ -5824,7 +5888,7 @@
         <v>9.6000000000000002E-2</v>
       </c>
     </row>
-    <row r="150" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:9">
       <c r="A150" s="2" t="s">
         <v>173</v>
       </c>
@@ -5853,7 +5917,7 @@
         <v>9.6000000000000002E-2</v>
       </c>
     </row>
-    <row r="151" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:9">
       <c r="A151" s="2" t="s">
         <v>174</v>
       </c>
@@ -5882,7 +5946,7 @@
         <v>9.0999999999999998E-2</v>
       </c>
     </row>
-    <row r="152" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:9">
       <c r="A152" s="2" t="s">
         <v>175</v>
       </c>
@@ -5911,7 +5975,7 @@
         <v>8.3000000000000004E-2</v>
       </c>
     </row>
-    <row r="153" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:9">
       <c r="A153" s="2" t="s">
         <v>176</v>
       </c>
@@ -5940,7 +6004,7 @@
         <v>8.1000000000000003E-2</v>
       </c>
     </row>
-    <row r="154" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:9">
       <c r="A154" s="1" t="s">
         <v>91</v>
       </c>
@@ -5969,7 +6033,7 @@
         <v>7.9000000000000001E-2</v>
       </c>
     </row>
-    <row r="155" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:9">
       <c r="A155" s="2" t="s">
         <v>177</v>
       </c>
@@ -5998,7 +6062,7 @@
         <v>7.9000000000000001E-2</v>
       </c>
     </row>
-    <row r="156" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:9">
       <c r="A156" s="2" t="s">
         <v>178</v>
       </c>
@@ -6027,7 +6091,7 @@
         <v>7.0999999999999994E-2</v>
       </c>
     </row>
-    <row r="157" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:9">
       <c r="A157" s="2" t="s">
         <v>179</v>
       </c>
@@ -6056,7 +6120,7 @@
         <v>6.9000000000000006E-2</v>
       </c>
     </row>
-    <row r="158" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:9">
       <c r="A158" s="2" t="s">
         <v>180</v>
       </c>
@@ -6085,7 +6149,7 @@
         <v>6.7000000000000004E-2</v>
       </c>
     </row>
-    <row r="159" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:9">
       <c r="A159" s="2" t="s">
         <v>181</v>
       </c>
@@ -6114,7 +6178,7 @@
         <v>6.7000000000000004E-2</v>
       </c>
     </row>
-    <row r="160" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:9">
       <c r="A160" s="2" t="s">
         <v>182</v>
       </c>
@@ -6143,7 +6207,7 @@
         <v>5.8999999999999997E-2</v>
       </c>
     </row>
-    <row r="161" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="161" spans="1:9">
       <c r="A161" s="1" t="s">
         <v>92</v>
       </c>
@@ -6172,7 +6236,7 @@
         <v>5.7000000000000002E-2</v>
       </c>
     </row>
-    <row r="162" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="162" spans="1:9">
       <c r="A162" s="2" t="s">
         <v>183</v>
       </c>
@@ -6201,7 +6265,7 @@
         <v>5.7000000000000002E-2</v>
       </c>
     </row>
-    <row r="163" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="163" spans="1:9">
       <c r="A163" s="1" t="s">
         <v>93</v>
       </c>
@@ -6230,7 +6294,7 @@
         <v>5.6000000000000001E-2</v>
       </c>
     </row>
-    <row r="164" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="164" spans="1:9">
       <c r="A164" s="1" t="s">
         <v>94</v>
       </c>
@@ -6259,7 +6323,7 @@
         <v>4.3999999999999997E-2</v>
       </c>
     </row>
-    <row r="165" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="165" spans="1:9">
       <c r="A165" s="2" t="s">
         <v>184</v>
       </c>
@@ -6288,7 +6352,7 @@
         <v>3.5999999999999997E-2</v>
       </c>
     </row>
-    <row r="166" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="166" spans="1:9">
       <c r="A166" s="2" t="s">
         <v>185</v>
       </c>
@@ -6317,7 +6381,7 @@
         <v>3.5999999999999997E-2</v>
       </c>
     </row>
-    <row r="167" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="167" spans="1:9">
       <c r="A167" s="2" t="s">
         <v>186</v>
       </c>
@@ -6346,7 +6410,7 @@
         <v>3.5999999999999997E-2</v>
       </c>
     </row>
-    <row r="168" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="168" spans="1:9">
       <c r="A168" s="1" t="s">
         <v>95</v>
       </c>
@@ -6375,7 +6439,7 @@
         <v>3.3000000000000002E-2</v>
       </c>
     </row>
-    <row r="169" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="169" spans="1:9">
       <c r="A169" s="2" t="s">
         <v>187</v>
       </c>
@@ -6404,7 +6468,7 @@
         <v>3.1E-2</v>
       </c>
     </row>
-    <row r="170" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="170" spans="1:9">
       <c r="A170" s="2" t="s">
         <v>188</v>
       </c>
@@ -6433,7 +6497,7 @@
         <v>3.1E-2</v>
       </c>
     </row>
-    <row r="171" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="171" spans="1:9">
       <c r="A171" s="1" t="s">
         <v>96</v>
       </c>
@@ -6462,7 +6526,7 @@
         <v>2.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="172" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="172" spans="1:9">
       <c r="A172" s="2" t="s">
         <v>189</v>
       </c>
@@ -6491,7 +6555,7 @@
         <v>2.4E-2</v>
       </c>
     </row>
-    <row r="173" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="173" spans="1:9">
       <c r="A173" s="1" t="s">
         <v>97</v>
       </c>
@@ -6520,7 +6584,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="174" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="174" spans="1:9">
       <c r="A174" s="2" t="s">
         <v>190</v>
       </c>
@@ -6549,7 +6613,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="175" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="175" spans="1:9">
       <c r="A175" s="1" t="s">
         <v>98</v>
       </c>
@@ -6578,7 +6642,7 @@
         <v>1.2999999999999999E-2</v>
       </c>
     </row>
-    <row r="176" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="176" spans="1:9">
       <c r="A176" s="2" t="s">
         <v>191</v>
       </c>
@@ -6607,7 +6671,7 @@
         <v>1.2999999999999999E-2</v>
       </c>
     </row>
-    <row r="177" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="177" spans="1:9">
       <c r="A177" s="2" t="s">
         <v>192</v>
       </c>
@@ -6636,7 +6700,7 @@
         <v>1.2999999999999999E-2</v>
       </c>
     </row>
-    <row r="178" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="178" spans="1:9">
       <c r="A178" s="1" t="s">
         <v>99</v>
       </c>
@@ -6665,7 +6729,7 @@
         <v>1.2E-2</v>
       </c>
     </row>
-    <row r="179" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="179" spans="1:9">
       <c r="A179" s="1" t="s">
         <v>100</v>
       </c>
@@ -6694,7 +6758,7 @@
         <v>8.0000000000000002E-3</v>
       </c>
     </row>
-    <row r="180" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="180" spans="1:9">
       <c r="A180" s="2" t="s">
         <v>193</v>
       </c>
@@ -6723,7 +6787,7 @@
         <v>7.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="181" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="181" spans="1:9">
       <c r="A181" s="1" t="s">
         <v>101</v>
       </c>
@@ -6752,7 +6816,7 @@
         <v>6.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="182" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="182" spans="1:9">
       <c r="A182" s="1" t="s">
         <v>102</v>
       </c>
@@ -6781,7 +6845,7 @@
         <v>3.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="183" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="183" spans="1:9">
       <c r="A183" s="1" t="s">
         <v>103</v>
       </c>
@@ -6810,7 +6874,7 @@
         <v>1E-3</v>
       </c>
     </row>
-    <row r="184" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="184" spans="1:9">
       <c r="A184" s="1" t="s">
         <v>104</v>
       </c>
@@ -6853,158 +6917,158 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{92BA6815-4D81-A240-B4E1-953F878982F1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{92BA6815-4D81-A240-B4E1-953F878982F1}">
   <dimension ref="A1:A30"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:1">
       <c r="A1" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1">
+      <c r="A2" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+    <row r="3" spans="1:1">
+      <c r="A3" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+    <row r="4" spans="1:1">
+      <c r="A4" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
+    <row r="5" spans="1:1">
+      <c r="A5" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
+    <row r="6" spans="1:1">
+      <c r="A6" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
+    <row r="7" spans="1:1">
+      <c r="A7" t="s">
         <v>206</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
+    <row r="8" spans="1:1">
+      <c r="A8" t="s">
         <v>207</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
+    <row r="9" spans="1:1">
+      <c r="A9" t="s">
         <v>208</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
+    <row r="10" spans="1:1">
+      <c r="A10" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
+    <row r="11" spans="1:1">
+      <c r="A11" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
+    <row r="12" spans="1:1">
+      <c r="A12" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
+    <row r="13" spans="1:1">
+      <c r="A13" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
+    <row r="14" spans="1:1">
+      <c r="A14" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
+    <row r="15" spans="1:1">
+      <c r="A15" t="s">
         <v>214</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
+    <row r="16" spans="1:1">
+      <c r="A16" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A16" t="s">
+    <row r="17" spans="1:1">
+      <c r="A17" t="s">
         <v>216</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
+    <row r="18" spans="1:1">
+      <c r="A18" t="s">
         <v>217</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
+    <row r="19" spans="1:1">
+      <c r="A19" t="s">
         <v>218</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A19" t="s">
+    <row r="20" spans="1:1">
+      <c r="A20" t="s">
         <v>219</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
+    <row r="21" spans="1:1">
+      <c r="A21" t="s">
         <v>220</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
+    <row r="22" spans="1:1">
+      <c r="A22" t="s">
         <v>221</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A22" t="s">
+    <row r="23" spans="1:1">
+      <c r="A23" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A23" t="s">
+    <row r="24" spans="1:1">
+      <c r="A24" t="s">
         <v>223</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A24" t="s">
+    <row r="25" spans="1:1">
+      <c r="A25" t="s">
         <v>224</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A25" t="s">
+    <row r="26" spans="1:1">
+      <c r="A26" t="s">
         <v>225</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A26" t="s">
+    <row r="27" spans="1:1">
+      <c r="A27" t="s">
         <v>226</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A27" t="s">
+    <row r="28" spans="1:1">
+      <c r="A28" t="s">
         <v>227</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A28" t="s">
+    <row r="29" spans="1:1">
+      <c r="A29" t="s">
         <v>228</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A29" t="s">
+    <row r="30" spans="1:1">
+      <c r="A30" t="s">
         <v>229</v>
-      </c>
-    </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A30" t="s">
-        <v>230</v>
       </c>
     </row>
   </sheetData>

</xml_diff>